<commit_message>
WIP: regen template/export Excel + nilai_ekonomi + site config & bantuan
database/template-import-export: regen 16 template xlsx + 16 export xlsx (2026-09-29) + 33 export CSV; tambah nilai_ekonomi.csv (template+export); generate-templates.mjs diperbarui.

src/config/site.ts + src/pages/government-assistance.tsx: perubahan WIP sesi sebelumnya (bantuan/site config).
</commit_message>
<xml_diff>
--- a/database/template-import-export/templates/template-ekonomi.xlsx
+++ b/database/template-import-export/templates/template-ekonomi.xlsx
@@ -9,13 +9,15 @@
     <sheet sheetId="3" name="CONTOH Inflasi" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Pasar" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="CONTOH Pasar" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Nilai Ekonomi" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="CONTOH Nilai Ekonomi" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="58">
   <si>
     <t/>
   </si>
@@ -23,10 +25,10 @@
     <t>EKONOMI</t>
   </si>
   <si>
-    <t>Inflasi tahunan (wilayah) dan jumlah pasar per jenis.</t>
-  </si>
-  <si>
-    <t>Dibuat otomatis: 22/9/2026, 14.21.33</t>
+    <t>Inflasi tahunan, jumlah pasar, dan nilai ekonomi bidang (input Dinas — tahunan/triwulan; semester = gabungan triwulan).</t>
+  </si>
+  <si>
+    <t>Dibuat otomatis: 29/9/2026, 15.29.43</t>
   </si>
   <si>
     <t>CARA PAKAI</t>
@@ -110,6 +112,36 @@
     <t>Jumlah Unit</t>
   </si>
   <si>
+    <t>Sheet "Nilai Ekonomi" — tabel nilai_ekonomi_tahunan</t>
+  </si>
+  <si>
+    <t>Bidang + Komoditas + Tahun + Triwulan (1-4; kosong = tahunan)</t>
+  </si>
+  <si>
+    <t>Bidang *</t>
+  </si>
+  <si>
+    <t>pilihan: pangan / hortikultura / perkebunan / peternakan / perikanan</t>
+  </si>
+  <si>
+    <t>Komoditas *</t>
+  </si>
+  <si>
+    <t>Satuan *</t>
+  </si>
+  <si>
+    <t>Triwulan (1-4; kosong = tahunan)</t>
+  </si>
+  <si>
+    <t>pilihan: 1 / 2 / 3 / 4</t>
+  </si>
+  <si>
+    <t>Volume *</t>
+  </si>
+  <si>
+    <t>Harga Produsen (Rp) *</t>
+  </si>
+  <si>
     <t>Wilayah</t>
   </si>
   <si>
@@ -132,6 +164,33 @@
   </si>
   <si>
     <t>Buah</t>
+  </si>
+  <si>
+    <t>Bidang</t>
+  </si>
+  <si>
+    <t>Komoditas</t>
+  </si>
+  <si>
+    <t>Satuan</t>
+  </si>
+  <si>
+    <t>Volume</t>
+  </si>
+  <si>
+    <t>Harga Produsen (Rp)</t>
+  </si>
+  <si>
+    <t>pangan</t>
+  </si>
+  <si>
+    <t>Contoh Komoditas</t>
+  </si>
+  <si>
+    <t>Contoh Satuan</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
 </sst>
 </file>
@@ -568,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -846,6 +905,132 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>0</v>
       </c>
     </row>
@@ -866,10 +1051,10 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>25</v>
@@ -888,10 +1073,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>25</v>
@@ -899,7 +1084,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B2">
         <v>2018</v>
@@ -910,7 +1095,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B3">
         <v>2018</v>
@@ -921,7 +1106,7 @@
     </row>
     <row r="5" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -941,10 +1126,10 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>30</v>
@@ -963,10 +1148,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>30</v>
@@ -974,7 +1159,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B2">
         <v>2016</v>
@@ -985,7 +1170,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B3">
         <v>2016</v>
@@ -996,7 +1181,117 @@
     </row>
     <row r="5" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>35</v>
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A2001">
+      <formula1>"pangan,hortikultura,perkebunan,peternakan,perikanan"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E2001">
+      <formula1>"1,2,3,4"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2">
+        <v>2025</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>